<commit_message>
Fix: Add Bentley's only to Thursday columns without affecting other days
- Uses empty row 22 for Bentley's (only N, O, P columns)
- Updated Daily Total formula to include P22
- Friday and all other day columns unchanged
</commit_message>
<xml_diff>
--- a/data/template_bag_count.xlsx
+++ b/data/template_bag_count.xlsx
@@ -910,7 +910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:T42"/>
+  <dimension ref="B2:T40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.85546875" customWidth="1" min="2" max="2"/>
@@ -1547,267 +1547,258 @@
       <c r="P22" s="16" t="n"/>
     </row>
     <row r="23" ht="15.75" customHeight="1" thickBot="1">
-      <c r="N23" s="39" t="n"/>
-      <c r="O23" s="11" t="n"/>
-      <c r="P23" s="10">
-        <f>P22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" thickBot="1"/>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>Superior Manor</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>Hall 100</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="n"/>
+      <c r="J23" s="28" t="inlineStr">
+        <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="K23" s="27" t="n"/>
+      <c r="L23" s="26" t="n"/>
+      <c r="N23" s="36" t="inlineStr">
+        <is>
+          <t>Daily Total Census</t>
+        </is>
+      </c>
+      <c r="P23">
+        <f>SUM(P8,P10,P14,P21,P22)</f>
+        <v/>
+      </c>
+      <c r="R23" s="18" t="inlineStr">
+        <is>
+          <t>Oakdale RCF</t>
+        </is>
+      </c>
+      <c r="S23" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="T23" s="16" t="n"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" thickBot="1">
+      <c r="B24" s="37" t="n"/>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>Hall 200</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="n"/>
+      <c r="R24" s="37" t="n"/>
+      <c r="S24" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="T24" s="13" t="n"/>
+    </row>
     <row r="25" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B25" s="21" t="inlineStr">
-        <is>
-          <t>Superior Manor</t>
-        </is>
-      </c>
-      <c r="C25" s="17" t="inlineStr">
-        <is>
-          <t>Hall 100</t>
-        </is>
-      </c>
-      <c r="D25" s="16" t="n"/>
-      <c r="J25" s="28" t="inlineStr">
-        <is>
-          <t>Legacy</t>
-        </is>
-      </c>
-      <c r="K25" s="27" t="n"/>
-      <c r="L25" s="26" t="n"/>
-      <c r="N25" s="36" t="inlineStr">
-        <is>
-          <t>Daily Total Census</t>
-        </is>
-      </c>
-      <c r="P25">
-        <f>SUM(P8,P10,P14,P21,P23)</f>
-        <v/>
-      </c>
-      <c r="R25" s="18" t="inlineStr">
-        <is>
-          <t>Oakdale RCF</t>
-        </is>
-      </c>
-      <c r="S25" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="T25" s="16" t="n"/>
+      <c r="B25" s="37" t="n"/>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Hall 300</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="n"/>
+      <c r="J25" s="40" t="inlineStr">
+        <is>
+          <t>John Knox</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr">
+        <is>
+          <t>CSL</t>
+        </is>
+      </c>
+      <c r="L25" s="16" t="n"/>
+      <c r="R25" s="39" t="n"/>
+      <c r="S25" s="11" t="n"/>
+      <c r="T25" s="10">
+        <f>SUM(T23:T24)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="37" t="n"/>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>Hall 200</t>
+          <t>Hall 400</t>
         </is>
       </c>
       <c r="D26" s="13" t="n"/>
-      <c r="R26" s="37" t="n"/>
-      <c r="S26" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="T26" s="13" t="n"/>
+      <c r="J26" s="37" t="n"/>
+      <c r="K26" s="14" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="L26" s="13" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B27" s="37" t="n"/>
-      <c r="C27" s="14" t="inlineStr">
-        <is>
-          <t>Hall 300</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="n"/>
-      <c r="J27" s="40" t="inlineStr">
-        <is>
-          <t>John Knox</t>
-        </is>
-      </c>
-      <c r="K27" s="17" t="inlineStr">
-        <is>
-          <t>CSL</t>
-        </is>
-      </c>
-      <c r="L27" s="16" t="n"/>
-      <c r="R27" s="39" t="n"/>
-      <c r="S27" s="11" t="n"/>
-      <c r="T27" s="10">
-        <f>SUM(T23:T24)</f>
+      <c r="B27" s="39" t="n"/>
+      <c r="C27" s="11" t="n"/>
+      <c r="D27" s="29">
+        <f>SUM(D23:D26)</f>
+        <v/>
+      </c>
+      <c r="J27" s="37" t="n"/>
+      <c r="K27" s="14" t="inlineStr">
+        <is>
+          <t>ALF</t>
+        </is>
+      </c>
+      <c r="L27" s="13" t="n"/>
+      <c r="R27" s="36" t="inlineStr">
+        <is>
+          <t>Daily Total Census</t>
+        </is>
+      </c>
+      <c r="T27">
+        <f>SUM(T4,T10,T16,T21,T25)</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B28" s="37" t="n"/>
-      <c r="C28" s="14" t="inlineStr">
-        <is>
-          <t>Hall 400</t>
-        </is>
-      </c>
-      <c r="D28" s="13" t="n"/>
       <c r="J28" s="37" t="n"/>
-      <c r="K28" s="14" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="L28" s="13" t="n"/>
+      <c r="K28" s="24" t="inlineStr">
+        <is>
+          <t>ILF 1</t>
+        </is>
+      </c>
+      <c r="L28" s="23" t="n"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B29" s="39" t="n"/>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="29">
-        <f>SUM(D23:D26)</f>
-        <v/>
-      </c>
+      <c r="B29" s="28" t="inlineStr">
+        <is>
+          <t>Walnut</t>
+        </is>
+      </c>
+      <c r="C29" s="27" t="n"/>
+      <c r="D29" s="26" t="n"/>
       <c r="J29" s="37" t="n"/>
-      <c r="K29" s="14" t="inlineStr">
+      <c r="K29" s="24" t="inlineStr">
+        <is>
+          <t>ILF 2</t>
+        </is>
+      </c>
+      <c r="L29" s="23" t="n"/>
+    </row>
+    <row r="30" ht="15.75" customHeight="1" thickBot="1">
+      <c r="J30" s="41" t="n"/>
+      <c r="K30" s="11" t="n"/>
+      <c r="L30" s="10">
+        <f>SUM(L25:L29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>Colonial Doniphan</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>Upstairs</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="n"/>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="B32" s="37" t="n"/>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="n"/>
+      <c r="J32" s="36" t="inlineStr">
+        <is>
+          <t>Daily Total Census</t>
+        </is>
+      </c>
+      <c r="L32">
+        <f>SUM(L4,L10,L15,L21,L23,L30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1" thickBot="1">
+      <c r="B33" s="39" t="n"/>
+      <c r="C33" s="11" t="n"/>
+      <c r="D33" s="10">
+        <f>SUM(D31:D32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1" thickBot="1"/>
+    <row r="35" ht="15" customHeight="1">
+      <c r="B35" s="18" t="inlineStr">
+        <is>
+          <t>New Hope</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
         <is>
           <t>ALF</t>
         </is>
       </c>
-      <c r="L29" s="13" t="n"/>
-      <c r="R29" s="36" t="inlineStr">
+      <c r="D35" s="16" t="n"/>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="B36" s="37" t="n"/>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>ILF</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="n"/>
+    </row>
+    <row r="37" ht="15.75" customHeight="1" thickBot="1">
+      <c r="B37" s="39" t="n"/>
+      <c r="C37" s="11" t="n"/>
+      <c r="D37" s="10">
+        <f>SUM(D35:D36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1" thickBot="1"/>
+    <row r="39" ht="21.75" customHeight="1">
+      <c r="B39" s="36" t="inlineStr">
         <is>
           <t>Daily Total Census</t>
         </is>
       </c>
-      <c r="T29">
-        <f>SUM(T4,T10,T16,T21,T25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1" thickBot="1">
-      <c r="J30" s="37" t="n"/>
-      <c r="K30" s="24" t="inlineStr">
-        <is>
-          <t>ILF 1</t>
-        </is>
-      </c>
-      <c r="L30" s="23" t="n"/>
-    </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="B31" s="28" t="inlineStr">
-        <is>
-          <t>Walnut</t>
-        </is>
-      </c>
-      <c r="C31" s="27" t="n"/>
-      <c r="D31" s="26" t="n"/>
-      <c r="J31" s="37" t="n"/>
-      <c r="K31" s="24" t="inlineStr">
-        <is>
-          <t>ILF 2</t>
-        </is>
-      </c>
-      <c r="L31" s="23" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1">
-      <c r="J32" s="41" t="n"/>
-      <c r="K32" s="11" t="n"/>
-      <c r="L32" s="10">
-        <f>SUM(L25:L29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1" thickBot="1">
-      <c r="B33" s="21" t="inlineStr">
-        <is>
-          <t>Colonial Doniphan</t>
-        </is>
-      </c>
-      <c r="C33" s="17" t="inlineStr">
-        <is>
-          <t>Upstairs</t>
-        </is>
-      </c>
-      <c r="D33" s="16" t="n"/>
-    </row>
-    <row r="34" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B34" s="37" t="n"/>
-      <c r="C34" s="14" t="inlineStr">
-        <is>
-          <t>Down</t>
-        </is>
-      </c>
-      <c r="D34" s="13" t="n"/>
-      <c r="J34" s="36" t="inlineStr">
-        <is>
-          <t>Daily Total Census</t>
-        </is>
-      </c>
-      <c r="L34">
-        <f>SUM(L4,L10,L15,L21,L23,L30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="15" customHeight="1">
-      <c r="B35" s="39" t="n"/>
-      <c r="C35" s="11" t="n"/>
-      <c r="D35" s="10">
-        <f>SUM(D31:D32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1"/>
-    <row r="37" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B37" s="18" t="inlineStr">
-        <is>
-          <t>New Hope</t>
-        </is>
-      </c>
-      <c r="C37" s="17" t="inlineStr">
-        <is>
-          <t>ALF</t>
-        </is>
-      </c>
-      <c r="D37" s="16" t="n"/>
-    </row>
-    <row r="38" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B38" s="37" t="n"/>
-      <c r="C38" s="14" t="inlineStr">
-        <is>
-          <t>ILF</t>
-        </is>
-      </c>
-      <c r="D38" s="13" t="n"/>
-    </row>
-    <row r="39" ht="21.75" customHeight="1">
-      <c r="B39" s="39" t="n"/>
-      <c r="C39" s="11" t="n"/>
-      <c r="D39" s="10">
-        <f>SUM(D35:D36)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="21" customHeight="1" thickBot="1"/>
-    <row r="41">
-      <c r="B41" s="36" t="inlineStr">
-        <is>
-          <t>Daily Total Census</t>
-        </is>
-      </c>
-      <c r="D41">
+      <c r="D39">
         <f>SUM(D8,D12,D17,D21,D27,D29,D33,D37)</f>
         <v/>
       </c>
-      <c r="J41" s="42" t="inlineStr">
+      <c r="J39" s="42" t="inlineStr">
         <is>
           <t>Weekly Census Count</t>
         </is>
       </c>
-      <c r="K41" s="43" t="n"/>
-      <c r="L41" s="44">
+      <c r="K39" s="43" t="n"/>
+      <c r="L39" s="44">
         <f>SUM(D39,H18,L32,P23,T27)</f>
         <v/>
       </c>
-      <c r="M41" s="43" t="n"/>
-      <c r="N41" s="43" t="n"/>
-      <c r="O41" s="45" t="n"/>
-    </row>
-    <row r="42">
-      <c r="J42" s="46" t="n"/>
-      <c r="K42" s="35" t="n"/>
-      <c r="L42" s="35" t="n"/>
-      <c r="M42" s="35" t="n"/>
-      <c r="N42" s="35" t="n"/>
-      <c r="O42" s="47" t="n"/>
+      <c r="M39" s="43" t="n"/>
+      <c r="N39" s="43" t="n"/>
+      <c r="O39" s="45" t="n"/>
+    </row>
+    <row r="40" ht="21" customHeight="1" thickBot="1">
+      <c r="J40" s="46" t="n"/>
+      <c r="K40" s="35" t="n"/>
+      <c r="L40" s="35" t="n"/>
+      <c r="M40" s="35" t="n"/>
+      <c r="N40" s="35" t="n"/>
+      <c r="O40" s="47" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="41">
@@ -1864,7 +1855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:T42"/>
+  <dimension ref="B2:T40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.85546875" customWidth="1" min="2" max="2"/>
@@ -2501,267 +2492,258 @@
       <c r="P22" s="16" t="n"/>
     </row>
     <row r="23" ht="15.75" customHeight="1" thickBot="1">
-      <c r="N23" s="39" t="n"/>
-      <c r="O23" s="11" t="n"/>
-      <c r="P23" s="10">
-        <f>P22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" thickBot="1"/>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>Superior Manor</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>Hall 100</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="n"/>
+      <c r="J23" s="28" t="inlineStr">
+        <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="K23" s="27" t="n"/>
+      <c r="L23" s="26" t="n"/>
+      <c r="N23" s="36" t="inlineStr">
+        <is>
+          <t>Daily Total Bags</t>
+        </is>
+      </c>
+      <c r="P23">
+        <f>SUM(P8,P10,P14,P21,P22)</f>
+        <v/>
+      </c>
+      <c r="R23" s="18" t="inlineStr">
+        <is>
+          <t>Oakdale RCF</t>
+        </is>
+      </c>
+      <c r="S23" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="T23" s="16" t="n"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" thickBot="1">
+      <c r="B24" s="37" t="n"/>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>Hall 200</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="n"/>
+      <c r="R24" s="37" t="n"/>
+      <c r="S24" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="T24" s="13" t="n"/>
+    </row>
     <row r="25" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B25" s="21" t="inlineStr">
-        <is>
-          <t>Superior Manor</t>
-        </is>
-      </c>
-      <c r="C25" s="17" t="inlineStr">
-        <is>
-          <t>Hall 100</t>
-        </is>
-      </c>
-      <c r="D25" s="16" t="n"/>
-      <c r="J25" s="28" t="inlineStr">
-        <is>
-          <t>Legacy</t>
-        </is>
-      </c>
-      <c r="K25" s="27" t="n"/>
-      <c r="L25" s="26" t="n"/>
-      <c r="N25" s="36" t="inlineStr">
-        <is>
-          <t>Daily Total Bags</t>
-        </is>
-      </c>
-      <c r="P25">
-        <f>SUM(P8,P10,P14,P21,P23)</f>
-        <v/>
-      </c>
-      <c r="R25" s="18" t="inlineStr">
-        <is>
-          <t>Oakdale RCF</t>
-        </is>
-      </c>
-      <c r="S25" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="T25" s="16" t="n"/>
+      <c r="B25" s="37" t="n"/>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Hall 300</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="n"/>
+      <c r="J25" s="40" t="inlineStr">
+        <is>
+          <t>John Knox</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr">
+        <is>
+          <t>CSL</t>
+        </is>
+      </c>
+      <c r="L25" s="16" t="n"/>
+      <c r="R25" s="39" t="n"/>
+      <c r="S25" s="11" t="n"/>
+      <c r="T25" s="10">
+        <f>SUM(T23:T24)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="37" t="n"/>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>Hall 200</t>
+          <t>Hall 400</t>
         </is>
       </c>
       <c r="D26" s="13" t="n"/>
-      <c r="R26" s="37" t="n"/>
-      <c r="S26" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="T26" s="13" t="n"/>
+      <c r="J26" s="37" t="n"/>
+      <c r="K26" s="14" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="L26" s="13" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B27" s="37" t="n"/>
-      <c r="C27" s="14" t="inlineStr">
-        <is>
-          <t>Hall 300</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="n"/>
-      <c r="J27" s="40" t="inlineStr">
-        <is>
-          <t>John Knox</t>
-        </is>
-      </c>
-      <c r="K27" s="17" t="inlineStr">
-        <is>
-          <t>CSL</t>
-        </is>
-      </c>
-      <c r="L27" s="16" t="n"/>
-      <c r="R27" s="39" t="n"/>
-      <c r="S27" s="11" t="n"/>
-      <c r="T27" s="10">
-        <f>SUM(T23:T24)</f>
+      <c r="B27" s="39" t="n"/>
+      <c r="C27" s="11" t="n"/>
+      <c r="D27" s="29">
+        <f>SUM(D23:D26)</f>
+        <v/>
+      </c>
+      <c r="J27" s="37" t="n"/>
+      <c r="K27" s="14" t="inlineStr">
+        <is>
+          <t>ALF</t>
+        </is>
+      </c>
+      <c r="L27" s="13" t="n"/>
+      <c r="R27" s="36" t="inlineStr">
+        <is>
+          <t>Daily Total Bags</t>
+        </is>
+      </c>
+      <c r="T27">
+        <f>SUM(T4,T10,T16,T21,T25)</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B28" s="37" t="n"/>
-      <c r="C28" s="14" t="inlineStr">
-        <is>
-          <t>Hall 400</t>
-        </is>
-      </c>
-      <c r="D28" s="13" t="n"/>
       <c r="J28" s="37" t="n"/>
-      <c r="K28" s="14" t="inlineStr">
-        <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="L28" s="13" t="n"/>
+      <c r="K28" s="24" t="inlineStr">
+        <is>
+          <t>ILF 1</t>
+        </is>
+      </c>
+      <c r="L28" s="23" t="n"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B29" s="39" t="n"/>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="29">
-        <f>SUM(D23:D26)</f>
-        <v/>
-      </c>
+      <c r="B29" s="28" t="inlineStr">
+        <is>
+          <t>Walnut</t>
+        </is>
+      </c>
+      <c r="C29" s="27" t="n"/>
+      <c r="D29" s="26" t="n"/>
       <c r="J29" s="37" t="n"/>
-      <c r="K29" s="14" t="inlineStr">
+      <c r="K29" s="24" t="inlineStr">
+        <is>
+          <t>ILF 2</t>
+        </is>
+      </c>
+      <c r="L29" s="23" t="n"/>
+    </row>
+    <row r="30" ht="15.75" customHeight="1" thickBot="1">
+      <c r="J30" s="41" t="n"/>
+      <c r="K30" s="11" t="n"/>
+      <c r="L30" s="10">
+        <f>SUM(L25:L29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>Colonial Doniphan</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>Upstairs</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="n"/>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="B32" s="37" t="n"/>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="n"/>
+      <c r="J32" s="36" t="inlineStr">
+        <is>
+          <t>Daily Total Bags</t>
+        </is>
+      </c>
+      <c r="L32">
+        <f>SUM(L4,L10,L15,L21,L23,L30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1" thickBot="1">
+      <c r="B33" s="39" t="n"/>
+      <c r="C33" s="11" t="n"/>
+      <c r="D33" s="10">
+        <f>SUM(D31:D32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1" thickBot="1"/>
+    <row r="35" ht="15" customHeight="1">
+      <c r="B35" s="18" t="inlineStr">
+        <is>
+          <t>New Hope</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
         <is>
           <t>ALF</t>
         </is>
       </c>
-      <c r="L29" s="13" t="n"/>
-      <c r="R29" s="36" t="inlineStr">
+      <c r="D35" s="16" t="n"/>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="B36" s="37" t="n"/>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>ILF</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="n"/>
+    </row>
+    <row r="37" ht="15.75" customHeight="1" thickBot="1">
+      <c r="B37" s="39" t="n"/>
+      <c r="C37" s="11" t="n"/>
+      <c r="D37" s="10">
+        <f>SUM(D35:D36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1" thickBot="1"/>
+    <row r="39" ht="21.75" customHeight="1">
+      <c r="B39" s="36" t="inlineStr">
         <is>
           <t>Daily Total Bags</t>
         </is>
       </c>
-      <c r="T29">
-        <f>SUM(T4,T10,T16,T21,T25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1" thickBot="1">
-      <c r="J30" s="37" t="n"/>
-      <c r="K30" s="24" t="inlineStr">
-        <is>
-          <t>ILF 1</t>
-        </is>
-      </c>
-      <c r="L30" s="23" t="n"/>
-    </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="B31" s="28" t="inlineStr">
-        <is>
-          <t>Walnut</t>
-        </is>
-      </c>
-      <c r="C31" s="27" t="n"/>
-      <c r="D31" s="26" t="n"/>
-      <c r="J31" s="37" t="n"/>
-      <c r="K31" s="24" t="inlineStr">
-        <is>
-          <t>ILF 2</t>
-        </is>
-      </c>
-      <c r="L31" s="23" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1">
-      <c r="J32" s="41" t="n"/>
-      <c r="K32" s="11" t="n"/>
-      <c r="L32" s="10">
-        <f>SUM(L25:L29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1" thickBot="1">
-      <c r="B33" s="21" t="inlineStr">
-        <is>
-          <t>Colonial Doniphan</t>
-        </is>
-      </c>
-      <c r="C33" s="17" t="inlineStr">
-        <is>
-          <t>Upstairs</t>
-        </is>
-      </c>
-      <c r="D33" s="16" t="n"/>
-    </row>
-    <row r="34" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B34" s="37" t="n"/>
-      <c r="C34" s="14" t="inlineStr">
-        <is>
-          <t>Down</t>
-        </is>
-      </c>
-      <c r="D34" s="13" t="n"/>
-      <c r="J34" s="36" t="inlineStr">
-        <is>
-          <t>Daily Total Bags</t>
-        </is>
-      </c>
-      <c r="L34">
-        <f>SUM(L4,L10,L15,L21,L23,L30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="15" customHeight="1">
-      <c r="B35" s="39" t="n"/>
-      <c r="C35" s="11" t="n"/>
-      <c r="D35" s="10">
-        <f>SUM(D31:D32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1"/>
-    <row r="37" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B37" s="18" t="inlineStr">
-        <is>
-          <t>New Hope</t>
-        </is>
-      </c>
-      <c r="C37" s="17" t="inlineStr">
-        <is>
-          <t>ALF</t>
-        </is>
-      </c>
-      <c r="D37" s="16" t="n"/>
-    </row>
-    <row r="38" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B38" s="37" t="n"/>
-      <c r="C38" s="14" t="inlineStr">
-        <is>
-          <t>ILF</t>
-        </is>
-      </c>
-      <c r="D38" s="13" t="n"/>
-    </row>
-    <row r="39" ht="21.75" customHeight="1">
-      <c r="B39" s="39" t="n"/>
-      <c r="C39" s="11" t="n"/>
-      <c r="D39" s="10">
-        <f>SUM(D35:D36)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="21" customHeight="1" thickBot="1"/>
-    <row r="41">
-      <c r="B41" s="36" t="inlineStr">
-        <is>
-          <t>Daily Total Bags</t>
-        </is>
-      </c>
-      <c r="D41">
+      <c r="D39">
         <f>SUM(D8,D12,D17,D21,D27,D29,D33,D37)</f>
         <v/>
       </c>
-      <c r="J41" s="42" t="inlineStr">
+      <c r="J39" s="42" t="inlineStr">
         <is>
           <t>Weekly Bag Count</t>
         </is>
       </c>
-      <c r="K41" s="43" t="n"/>
-      <c r="L41" s="44">
+      <c r="K39" s="43" t="n"/>
+      <c r="L39" s="44">
         <f>SUM(D39,H18,L32,P23,T27)</f>
         <v/>
       </c>
-      <c r="M41" s="43" t="n"/>
-      <c r="N41" s="43" t="n"/>
-      <c r="O41" s="45" t="n"/>
-    </row>
-    <row r="42">
-      <c r="J42" s="46" t="n"/>
-      <c r="K42" s="35" t="n"/>
-      <c r="L42" s="35" t="n"/>
-      <c r="M42" s="35" t="n"/>
-      <c r="N42" s="35" t="n"/>
-      <c r="O42" s="47" t="n"/>
+      <c r="M39" s="43" t="n"/>
+      <c r="N39" s="43" t="n"/>
+      <c r="O39" s="45" t="n"/>
+    </row>
+    <row r="40" ht="21" customHeight="1" thickBot="1">
+      <c r="J40" s="46" t="n"/>
+      <c r="K40" s="35" t="n"/>
+      <c r="L40" s="35" t="n"/>
+      <c r="M40" s="35" t="n"/>
+      <c r="N40" s="35" t="n"/>
+      <c r="O40" s="47" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="41">

</xml_diff>

<commit_message>
Add Bentley's with proper spacing in Thursday column only
- Row 22: blank (space after U-City)
- Row 23: Bentley's facility
- Row 24: Bentley's total
- Row 25: blank (space before daily total)
- Row 26: Daily Total (shifted down, formula updated)
- Other day columns unchanged
</commit_message>
<xml_diff>
--- a/data/template_bag_count.xlsx
+++ b/data/template_bag_count.xlsx
@@ -1533,19 +1533,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1" thickBot="1">
-      <c r="N22" s="18" t="inlineStr">
-        <is>
-          <t>Bentley's</t>
-        </is>
-      </c>
-      <c r="O22" s="17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="P22" s="16" t="n"/>
-    </row>
+    <row r="22" ht="15.75" customHeight="1" thickBot="1"/>
     <row r="23" ht="15.75" customHeight="1" thickBot="1">
       <c r="B23" s="21" t="inlineStr">
         <is>
@@ -1565,15 +1553,17 @@
       </c>
       <c r="K23" s="27" t="n"/>
       <c r="L23" s="26" t="n"/>
-      <c r="N23" s="36" t="inlineStr">
-        <is>
-          <t>Daily Total Census</t>
-        </is>
-      </c>
-      <c r="P23">
-        <f>SUM(P8,P10,P14,P21,P22)</f>
-        <v/>
-      </c>
+      <c r="N23" s="18" t="inlineStr">
+        <is>
+          <t>Bentley's</t>
+        </is>
+      </c>
+      <c r="O23" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P23" s="16" t="n"/>
       <c r="R23" s="18" t="inlineStr">
         <is>
           <t>Oakdale RCF</t>
@@ -1592,6 +1582,12 @@
         </is>
       </c>
       <c r="D24" s="13" t="n"/>
+      <c r="N24" s="39" t="n"/>
+      <c r="O24" s="11" t="n"/>
+      <c r="P24" s="10">
+        <f>P23</f>
+        <v/>
+      </c>
       <c r="R24" s="37" t="n"/>
       <c r="S24" s="14" t="n">
         <v>2</v>
@@ -1639,6 +1635,15 @@
         </is>
       </c>
       <c r="L26" s="13" t="n"/>
+      <c r="N26" s="36" t="inlineStr">
+        <is>
+          <t>Daily Total Census</t>
+        </is>
+      </c>
+      <c r="P26">
+        <f>SUM(P8,P10,P14,P21,P24)</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" thickBot="1">
       <c r="B27" s="39" t="n"/>
@@ -1801,7 +1806,7 @@
       <c r="O40" s="47" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="41">
+  <mergeCells count="40">
     <mergeCell ref="R12:R16"/>
     <mergeCell ref="F4:F7"/>
     <mergeCell ref="C4:C5"/>
@@ -1819,7 +1824,6 @@
     <mergeCell ref="B19:B21"/>
     <mergeCell ref="R27:S27"/>
     <mergeCell ref="S6:S7"/>
-    <mergeCell ref="N23:O23"/>
     <mergeCell ref="L39:O40"/>
     <mergeCell ref="R23:R25"/>
     <mergeCell ref="J17:J21"/>
@@ -2478,19 +2482,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1" thickBot="1">
-      <c r="N22" s="18" t="inlineStr">
-        <is>
-          <t>Bentley's</t>
-        </is>
-      </c>
-      <c r="O22" s="17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="P22" s="16" t="n"/>
-    </row>
+    <row r="22" ht="15.75" customHeight="1" thickBot="1"/>
     <row r="23" ht="15.75" customHeight="1" thickBot="1">
       <c r="B23" s="21" t="inlineStr">
         <is>
@@ -2510,15 +2502,17 @@
       </c>
       <c r="K23" s="27" t="n"/>
       <c r="L23" s="26" t="n"/>
-      <c r="N23" s="36" t="inlineStr">
-        <is>
-          <t>Daily Total Bags</t>
-        </is>
-      </c>
-      <c r="P23">
-        <f>SUM(P8,P10,P14,P21,P22)</f>
-        <v/>
-      </c>
+      <c r="N23" s="18" t="inlineStr">
+        <is>
+          <t>Bentley's</t>
+        </is>
+      </c>
+      <c r="O23" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P23" s="16" t="n"/>
       <c r="R23" s="18" t="inlineStr">
         <is>
           <t>Oakdale RCF</t>
@@ -2537,6 +2531,12 @@
         </is>
       </c>
       <c r="D24" s="13" t="n"/>
+      <c r="N24" s="39" t="n"/>
+      <c r="O24" s="11" t="n"/>
+      <c r="P24" s="10">
+        <f>P23</f>
+        <v/>
+      </c>
       <c r="R24" s="37" t="n"/>
       <c r="S24" s="14" t="n">
         <v>2</v>
@@ -2584,6 +2584,15 @@
         </is>
       </c>
       <c r="L26" s="13" t="n"/>
+      <c r="N26" s="36" t="inlineStr">
+        <is>
+          <t>Daily Total Bags</t>
+        </is>
+      </c>
+      <c r="P26">
+        <f>SUM(P8,P10,P14,P21,P24)</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" thickBot="1">
       <c r="B27" s="39" t="n"/>
@@ -2746,7 +2755,7 @@
       <c r="O40" s="47" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="41">
+  <mergeCells count="40">
     <mergeCell ref="R12:R16"/>
     <mergeCell ref="F4:F7"/>
     <mergeCell ref="C4:C5"/>
@@ -2763,7 +2772,6 @@
     <mergeCell ref="F18:G18"/>
     <mergeCell ref="B19:B21"/>
     <mergeCell ref="R27:S27"/>
-    <mergeCell ref="N23:O23"/>
     <mergeCell ref="S6:S7"/>
     <mergeCell ref="L39:O40"/>
     <mergeCell ref="R23:R25"/>

</xml_diff>